<commit_message>
Adding feature to run checklist in the others servers of data adquisition.
</commit_message>
<xml_diff>
--- a/data/siigeo_stations.xlsx
+++ b/data/siigeo_stations.xlsx
@@ -4036,7 +4036,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2023-02-20 13:00:00</t>
+          <t>2025-09-29 18:15:00</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
@@ -8542,12 +8542,12 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>CMG-5T, DC_100 s,  0.255 V/m/s**2, 4g clip level,</t>
+          <t>LK-307-115, DC to 200 Hz, 20Vp single-ended full s</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>2023-02-10 13:00:00</t>
+          <t>2025-09-30 18:39:00</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
@@ -8572,11 +8572,7 @@
         </is>
       </c>
       <c r="V63" s="2" t="inlineStr"/>
-      <c r="W63" s="2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
+      <c r="W63" s="2" t="inlineStr"/>
       <c r="X63" s="2" t="inlineStr">
         <is>
           <t>Permanente</t>
@@ -18151,7 +18147,7 @@
       </c>
       <c r="M138" s="2" t="inlineStr">
         <is>
-          <t>PAOLA ANDREA ATAPUMA</t>
+          <t>LUISA CASTILLO</t>
         </is>
       </c>
       <c r="N138" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Eliminating AUA1 and complete docstring for functions of network class.
</commit_message>
<xml_diff>
--- a/data/siigeo_stations.xlsx
+++ b/data/siigeo_stations.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>MIGUEL LIZARAZO</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>MIGUEL LIZARAZO</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>ANGEL DANIEL AGUDELO</t>
+          <t>HELBER GARCIA</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>ANGEL DANIEL AGUDELO</t>
+          <t>HELBER GARCIA</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>VIVIANA DIONICIO</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>VIVIANA DIONICIO</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>LUISA CASTILLO</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>VIVIANA DIONICIO</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>VIVIANA DIONICIO</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
@@ -11495,7 +11495,7 @@
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>VIVIANA DIONICIO</t>
         </is>
       </c>
       <c r="N86" s="2" t="inlineStr">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>PAOLA ANDREA ATAPUMA</t>
+          <t>ELIZABETH MAZO</t>
         </is>
       </c>
       <c r="N95" s="2" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>PAOLA ANDREA ATAPUMA</t>
+          <t>ELIZABETH MAZO</t>
         </is>
       </c>
       <c r="N96" s="2" t="inlineStr">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>PAOLA ANDREA ATAPUMA</t>
+          <t>ELIZABETH MAZO</t>
         </is>
       </c>
       <c r="N97" s="2" t="inlineStr">
@@ -13297,7 +13297,7 @@
       <c r="L100" s="2" t="inlineStr"/>
       <c r="M100" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N100" s="2" t="inlineStr">
@@ -13414,7 +13414,7 @@
       <c r="L101" s="2" t="inlineStr"/>
       <c r="M101" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N101" s="2" t="inlineStr">
@@ -13539,7 +13539,7 @@
       <c r="L102" s="2" t="inlineStr"/>
       <c r="M102" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N102" s="2" t="inlineStr">
@@ -13664,7 +13664,7 @@
       <c r="L103" s="2" t="inlineStr"/>
       <c r="M103" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N103" s="2" t="inlineStr">
@@ -13789,7 +13789,7 @@
       <c r="L104" s="2" t="inlineStr"/>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N104" s="2" t="inlineStr">
@@ -13914,7 +13914,7 @@
       <c r="L105" s="2" t="inlineStr"/>
       <c r="M105" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N105" s="2" t="inlineStr">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>MIGUEL LIZARAZO</t>
         </is>
       </c>
       <c r="N106" s="2" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="M122" s="2" t="inlineStr">
         <is>
-          <t>PAOLA ANDREA ATAPUMA</t>
+          <t>HELBER GARCIA</t>
         </is>
       </c>
       <c r="N122" s="2" t="inlineStr">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="M123" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N123" s="2" t="inlineStr">
@@ -16740,7 +16740,7 @@
       </c>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N127" s="2" t="inlineStr">
@@ -21743,7 +21743,7 @@
       <c r="L166" s="2" t="inlineStr"/>
       <c r="M166" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N166" s="2" t="inlineStr">
@@ -21868,7 +21868,7 @@
       <c r="L167" s="2" t="inlineStr"/>
       <c r="M167" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>DANIEL RUIZ</t>
         </is>
       </c>
       <c r="N167" s="2" t="inlineStr">
@@ -27004,7 +27004,7 @@
       </c>
       <c r="M207" s="2" t="inlineStr">
         <is>
-          <t>OMAR MERCADO</t>
+          <t>MIGUEL LIZARAZO</t>
         </is>
       </c>
       <c r="N207" s="2" t="inlineStr">

</xml_diff>